<commit_message>
editing with current tensile testing results
</commit_message>
<xml_diff>
--- a/tensile_strength_clammp.xlsx
+++ b/tensile_strength_clammp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nuwildcat-my.sharepoint.com/personal/stn424_ads_northwestern_edu/Documents/Collaborations/Proposals/GO-Barrier, TFMI Proposals with Tim Wei/URAP_2023-10/Shared/Lanning, Mackenzie/graphene-oxide-paper-coatings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="8_{E7047EFC-AC87-1446-9EE2-AFD11443121C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B449AC5C-D5B9-F249-8F15-DFA47597011A}"/>
+  <xr:revisionPtr revIDLastSave="222" documentId="8_{E7047EFC-AC87-1446-9EE2-AFD11443121C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6A37B31-4DC4-154E-AD19-E34238BB37FC}"/>
   <bookViews>
     <workbookView xWindow="1060" yWindow="1240" windowWidth="27640" windowHeight="16740" xr2:uid="{9D6F6D14-15C4-894F-A380-C8BF75B569C1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="19">
   <si>
     <t>Sample</t>
   </si>
@@ -484,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1161D6ED-F005-7245-AC8F-CA8CEF89B76D}">
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.33203125" customWidth="1"/>
@@ -2734,6 +2734,406 @@
         <v>183.21440100000001</v>
       </c>
     </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <v>1</v>
+      </c>
+      <c r="B113" t="s">
+        <v>6</v>
+      </c>
+      <c r="C113" t="s">
+        <v>17</v>
+      </c>
+      <c r="D113" t="s">
+        <v>16</v>
+      </c>
+      <c r="E113" t="s">
+        <v>9</v>
+      </c>
+      <c r="F113" s="2">
+        <v>52.606754000000002</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>2</v>
+      </c>
+      <c r="B114" t="s">
+        <v>6</v>
+      </c>
+      <c r="C114" t="s">
+        <v>17</v>
+      </c>
+      <c r="D114" t="s">
+        <v>16</v>
+      </c>
+      <c r="E114" t="s">
+        <v>9</v>
+      </c>
+      <c r="F114" s="2">
+        <v>66.542145000000005</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>3</v>
+      </c>
+      <c r="B115" t="s">
+        <v>6</v>
+      </c>
+      <c r="C115" t="s">
+        <v>17</v>
+      </c>
+      <c r="D115" t="s">
+        <v>16</v>
+      </c>
+      <c r="E115" t="s">
+        <v>9</v>
+      </c>
+      <c r="F115" s="2">
+        <v>67.156981999999999</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>4</v>
+      </c>
+      <c r="B116" t="s">
+        <v>6</v>
+      </c>
+      <c r="C116" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" t="s">
+        <v>16</v>
+      </c>
+      <c r="E116" t="s">
+        <v>9</v>
+      </c>
+      <c r="F116" s="2">
+        <v>65.702720999999997</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <v>5</v>
+      </c>
+      <c r="B117" t="s">
+        <v>6</v>
+      </c>
+      <c r="C117" t="s">
+        <v>17</v>
+      </c>
+      <c r="D117" t="s">
+        <v>16</v>
+      </c>
+      <c r="E117" t="s">
+        <v>9</v>
+      </c>
+      <c r="F117" s="2">
+        <v>79.301247000000004</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <v>6</v>
+      </c>
+      <c r="B118" t="s">
+        <v>6</v>
+      </c>
+      <c r="C118" t="s">
+        <v>17</v>
+      </c>
+      <c r="D118" t="s">
+        <v>16</v>
+      </c>
+      <c r="E118" t="s">
+        <v>9</v>
+      </c>
+      <c r="F118" s="2">
+        <v>70.130882</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <v>7</v>
+      </c>
+      <c r="B119" t="s">
+        <v>6</v>
+      </c>
+      <c r="C119" t="s">
+        <v>17</v>
+      </c>
+      <c r="D119" t="s">
+        <v>16</v>
+      </c>
+      <c r="E119" t="s">
+        <v>9</v>
+      </c>
+      <c r="F119" s="2">
+        <v>84.646827999999999</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <v>8</v>
+      </c>
+      <c r="B120" t="s">
+        <v>6</v>
+      </c>
+      <c r="C120" t="s">
+        <v>17</v>
+      </c>
+      <c r="D120" t="s">
+        <v>16</v>
+      </c>
+      <c r="E120" t="s">
+        <v>9</v>
+      </c>
+      <c r="F120" s="2">
+        <v>74.772796999999997</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>9</v>
+      </c>
+      <c r="B121" t="s">
+        <v>6</v>
+      </c>
+      <c r="C121" t="s">
+        <v>17</v>
+      </c>
+      <c r="D121" t="s">
+        <v>16</v>
+      </c>
+      <c r="E121" t="s">
+        <v>9</v>
+      </c>
+      <c r="F121" s="2">
+        <v>68.441779999999994</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>10</v>
+      </c>
+      <c r="B122" t="s">
+        <v>6</v>
+      </c>
+      <c r="C122" t="s">
+        <v>17</v>
+      </c>
+      <c r="D122" t="s">
+        <v>16</v>
+      </c>
+      <c r="E122" t="s">
+        <v>9</v>
+      </c>
+      <c r="F122" s="2">
+        <v>69.148674</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A123">
+        <v>1</v>
+      </c>
+      <c r="B123" t="s">
+        <v>6</v>
+      </c>
+      <c r="C123" t="s">
+        <v>18</v>
+      </c>
+      <c r="D123" t="s">
+        <v>16</v>
+      </c>
+      <c r="E123" t="s">
+        <v>9</v>
+      </c>
+      <c r="F123" s="2">
+        <v>68.045074</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A124">
+        <v>2</v>
+      </c>
+      <c r="B124" t="s">
+        <v>6</v>
+      </c>
+      <c r="C124" t="s">
+        <v>18</v>
+      </c>
+      <c r="D124" t="s">
+        <v>16</v>
+      </c>
+      <c r="E124" t="s">
+        <v>9</v>
+      </c>
+      <c r="F124" s="2">
+        <v>71.723831000000004</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A125">
+        <v>3</v>
+      </c>
+      <c r="B125" t="s">
+        <v>6</v>
+      </c>
+      <c r="C125" t="s">
+        <v>18</v>
+      </c>
+      <c r="D125" t="s">
+        <v>16</v>
+      </c>
+      <c r="E125" t="s">
+        <v>9</v>
+      </c>
+      <c r="F125" s="2">
+        <v>59.385185</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A126">
+        <v>4</v>
+      </c>
+      <c r="B126" t="s">
+        <v>6</v>
+      </c>
+      <c r="C126" t="s">
+        <v>18</v>
+      </c>
+      <c r="D126" t="s">
+        <v>16</v>
+      </c>
+      <c r="E126" t="s">
+        <v>9</v>
+      </c>
+      <c r="F126" s="2">
+        <v>69.775238000000002</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A127">
+        <v>5</v>
+      </c>
+      <c r="B127" t="s">
+        <v>6</v>
+      </c>
+      <c r="C127" t="s">
+        <v>18</v>
+      </c>
+      <c r="D127" t="s">
+        <v>16</v>
+      </c>
+      <c r="E127" t="s">
+        <v>9</v>
+      </c>
+      <c r="F127" s="2">
+        <v>76.287177999999997</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>6</v>
+      </c>
+      <c r="B128" t="s">
+        <v>6</v>
+      </c>
+      <c r="C128" t="s">
+        <v>18</v>
+      </c>
+      <c r="D128" t="s">
+        <v>16</v>
+      </c>
+      <c r="E128" t="s">
+        <v>9</v>
+      </c>
+      <c r="F128" s="2">
+        <v>69.871703999999994</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>7</v>
+      </c>
+      <c r="B129" t="s">
+        <v>6</v>
+      </c>
+      <c r="C129" t="s">
+        <v>18</v>
+      </c>
+      <c r="D129" t="s">
+        <v>16</v>
+      </c>
+      <c r="E129" t="s">
+        <v>9</v>
+      </c>
+      <c r="F129" s="2">
+        <v>64.807006999999999</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>8</v>
+      </c>
+      <c r="B130" t="s">
+        <v>6</v>
+      </c>
+      <c r="C130" t="s">
+        <v>18</v>
+      </c>
+      <c r="D130" t="s">
+        <v>16</v>
+      </c>
+      <c r="E130" t="s">
+        <v>9</v>
+      </c>
+      <c r="F130" s="2">
+        <v>58.587989999999998</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>9</v>
+      </c>
+      <c r="B131" t="s">
+        <v>6</v>
+      </c>
+      <c r="C131" t="s">
+        <v>18</v>
+      </c>
+      <c r="D131" t="s">
+        <v>16</v>
+      </c>
+      <c r="E131" t="s">
+        <v>9</v>
+      </c>
+      <c r="F131" s="2">
+        <v>74.616530999999995</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>10</v>
+      </c>
+      <c r="B132" t="s">
+        <v>6</v>
+      </c>
+      <c r="C132" t="s">
+        <v>18</v>
+      </c>
+      <c r="D132" t="s">
+        <v>16</v>
+      </c>
+      <c r="E132" t="s">
+        <v>9</v>
+      </c>
+      <c r="F132" s="2">
+        <v>63.845032000000003</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>